<commit_message>
First batch committed to JLC
</commit_message>
<xml_diff>
--- a/PCB/Gerbers/Twin_PLL_GPSDO-JLCPCB-CPL_v_1_1.xlsx
+++ b/PCB/Gerbers/Twin_PLL_GPSDO-JLCPCB-CPL_v_1_1.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E138"/>
+  <dimension ref="A1:E137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -635,17 +635,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C16</t>
+          <t>C17</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>44.4750mm</t>
+          <t>46.6975mm</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>20.0225mm</t>
+          <t>19.3875mm</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -662,17 +662,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C17</t>
+          <t>C18</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>46.6975mm</t>
+          <t>24.4475mm</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>19.3875mm</t>
+          <t>7.9375mm</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -682,24 +682,24 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>270</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C18</t>
+          <t>C19</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>24.4475mm</t>
+          <t>10.1600mm</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>7.9375mm</t>
+          <t>22.8600mm</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -709,24 +709,24 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>C19</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10.1600mm</t>
+          <t>82.1250mm</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>22.8600mm</t>
+          <t>10.2300mm</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -736,24 +736,24 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>C20</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>82.1250mm</t>
+          <t>10.1600mm</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>10.2300mm</t>
+          <t>25.0825mm</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -763,24 +763,24 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>C20</t>
+          <t>C21</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.1600mm</t>
+          <t>9.2075mm</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>25.0825mm</t>
+          <t>10.7950mm</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -790,19 +790,19 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>270</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>C21</t>
+          <t>C22</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>9.2075mm</t>
+          <t>11.4300mm</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -824,17 +824,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>C22</t>
+          <t>C23</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>11.4300mm</t>
+          <t>41.7842mm</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>10.7950mm</t>
+          <t>20.9951mm</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -844,24 +844,24 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>C23</t>
+          <t>C24</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>41.7842mm</t>
+          <t>66.1607mm</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>20.9951mm</t>
+          <t>7.0160mm</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -871,24 +871,24 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>270</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>C24</t>
+          <t>C25</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>66.1607mm</t>
+          <t>68.2141mm</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>7.0160mm</t>
+          <t>7.0272mm</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -905,17 +905,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>C25</t>
+          <t>C26</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>68.2141mm</t>
+          <t>72.3959mm</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>7.0272mm</t>
+          <t>39.6491mm</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -925,24 +925,24 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>C26</t>
+          <t>C27</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>72.3959mm</t>
+          <t>75.0073mm</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>39.6491mm</t>
+          <t>18.1588mm</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -952,24 +952,24 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>180</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>C27</t>
+          <t>C28</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>75.0073mm</t>
+          <t>20.9550mm</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>18.1588mm</t>
+          <t>7.9375mm</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -979,24 +979,24 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>270</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>C28</t>
+          <t>C29</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>20.9550mm</t>
+          <t>29.5275mm</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>7.9375mm</t>
+          <t>24.7650mm</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1006,24 +1006,24 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>180</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>C29</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>29.5275mm</t>
+          <t>80.2364mm</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>24.7650mm</t>
+          <t>10.2300mm</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1033,24 +1033,24 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>C30</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>80.2364mm</t>
+          <t>69.5032mm</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>10.2300mm</t>
+          <t>17.5365mm</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1060,24 +1060,24 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>C30</t>
+          <t>C31</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>69.5032mm</t>
+          <t>69.5113mm</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>17.5365mm</t>
+          <t>15.5050mm</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1094,17 +1094,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>C31</t>
+          <t>C32</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>69.5113mm</t>
+          <t>91.5750mm</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>15.5050mm</t>
+          <t>33.9700mm</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1114,24 +1114,24 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>C32</t>
+          <t>C33</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>91.5750mm</t>
+          <t>84.3450mm</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>33.9700mm</t>
+          <t>19.4500mm</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1141,24 +1141,24 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>270</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>C33</t>
+          <t>C34</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>84.3450mm</t>
+          <t>93.4028mm</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>19.4500mm</t>
+          <t>33.9700mm</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1168,24 +1168,24 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>C34</t>
+          <t>C35</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>93.4028mm</t>
+          <t>89.9553mm</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>33.9700mm</t>
+          <t>31.2598mm</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1202,17 +1202,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>C35</t>
+          <t>C36</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>89.9553mm</t>
+          <t>63.1803mm</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>31.2598mm</t>
+          <t>14.2384mm</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1229,17 +1229,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>C36</t>
+          <t>C37</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>63.1803mm</t>
+          <t>60.9240mm</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>14.2384mm</t>
+          <t>14.2356mm</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1256,17 +1256,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>C37</t>
+          <t>C38</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>60.9240mm</t>
+          <t>61.7982mm</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>14.2356mm</t>
+          <t>10.0076mm</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1276,24 +1276,24 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>C38</t>
+          <t>C39</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>61.7982mm</t>
+          <t>88.2600mm</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>10.0076mm</t>
+          <t>31.6900mm</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1303,24 +1303,24 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>C39</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>88.2600mm</t>
+          <t>89.9553mm</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>31.6900mm</t>
+          <t>7.2598mm</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1337,17 +1337,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C40</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>89.9553mm</t>
+          <t>92.2496mm</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>7.2598mm</t>
+          <t>40.6900mm</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1357,24 +1357,24 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>180</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>C40</t>
+          <t>C41</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>92.2496mm</t>
+          <t>95.3750mm</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>40.6900mm</t>
+          <t>42.4400mm</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1384,24 +1384,24 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>270</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>C41</t>
+          <t>C42</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>95.3750mm</t>
+          <t>90.8750mm</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>42.4400mm</t>
+          <t>43.4400mm</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1418,12 +1418,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>C42</t>
+          <t>C43</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>90.8750mm</t>
+          <t>92.5250mm</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1445,17 +1445,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>C43</t>
+          <t>C44</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>92.5250mm</t>
+          <t>81.2478mm</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>43.4400mm</t>
+          <t>20.2322mm</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1465,24 +1465,24 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>C44</t>
+          <t>C45</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>81.2478mm</t>
+          <t>84.3450mm</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>20.2322mm</t>
+          <t>43.4500mm</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1492,24 +1492,24 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>270</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>C45</t>
+          <t>C46</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>84.3450mm</t>
+          <t>81.2850mm</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>43.4500mm</t>
+          <t>16.9900mm</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1519,24 +1519,24 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>180</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>C46</t>
+          <t>C47</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>81.2850mm</t>
+          <t>81.2750mm</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>16.9900mm</t>
+          <t>18.5100mm</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1553,17 +1553,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>C47</t>
+          <t>C48</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>81.2750mm</t>
+          <t>95.3460mm</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>18.5100mm</t>
+          <t>8.7663mm</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1573,24 +1573,24 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>C48</t>
+          <t>C49</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>95.3460mm</t>
+          <t>98.2750mm</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>8.7663mm</t>
+          <t>17.1400mm</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1600,24 +1600,24 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>180</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>C49</t>
+          <t>C5</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>98.2750mm</t>
+          <t>88.2600mm</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>17.1400mm</t>
+          <t>7.6900mm</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1627,24 +1627,24 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>C5</t>
+          <t>C50</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>88.2600mm</t>
+          <t>100.1800mm</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>7.6900mm</t>
+          <t>21.3300mm</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1654,24 +1654,24 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>180</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>C50</t>
+          <t>C51</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>100.1800mm</t>
+          <t>100.1703mm</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>21.3300mm</t>
+          <t>23.3525mm</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1688,17 +1688,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>C51</t>
+          <t>C52</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>100.1703mm</t>
+          <t>71.9709mm</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>23.3525mm</t>
+          <t>24.7904mm</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1708,24 +1708,24 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>270</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>C52</t>
+          <t>C53</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>71.9709mm</t>
+          <t>98.2750mm</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>24.7904mm</t>
+          <t>14.4900mm</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1735,24 +1735,24 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>C53</t>
+          <t>C54</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>98.2750mm</t>
+          <t>87.6250mm</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>14.4900mm</t>
+          <t>22.5900mm</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1762,19 +1762,19 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>270</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>C54</t>
+          <t>C55</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>87.6250mm</t>
+          <t>89.2250mm</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1789,24 +1789,24 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>C55</t>
+          <t>C56</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>89.2250mm</t>
+          <t>87.6250mm</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>22.5900mm</t>
+          <t>19.4400mm</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1816,24 +1816,24 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>270</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>C56</t>
+          <t>C57</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>87.6250mm</t>
+          <t>81.2478mm</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>19.4400mm</t>
+          <t>44.2322mm</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1843,24 +1843,24 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>C57</t>
+          <t>C58</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>81.2478mm</t>
+          <t>81.2850mm</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>44.2322mm</t>
+          <t>40.9900mm</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1870,24 +1870,24 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>180</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>C58</t>
+          <t>C59</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>81.2850mm</t>
+          <t>81.2750mm</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>40.9900mm</t>
+          <t>42.5100mm</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1904,17 +1904,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>C59</t>
+          <t>C6</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>81.2750mm</t>
+          <t>82.0250mm</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>42.5100mm</t>
+          <t>14.4900mm</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1924,24 +1924,24 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>C60</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>82.0250mm</t>
+          <t>95.3968mm</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>14.4900mm</t>
+          <t>32.6520mm</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1958,17 +1958,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>C60</t>
+          <t>C61</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>95.3968mm</t>
+          <t>98.2750mm</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>32.6520mm</t>
+          <t>41.1400mm</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1978,24 +1978,24 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>180</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>C61</t>
+          <t>C62</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>98.2750mm</t>
+          <t>100.1800mm</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>41.1400mm</t>
+          <t>45.3300mm</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2012,17 +2012,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>C62</t>
+          <t>C63</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>100.1800mm</t>
+          <t>100.1703mm</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>45.3300mm</t>
+          <t>47.3525mm</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2039,17 +2039,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>C63</t>
+          <t>C64</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>100.1703mm</t>
+          <t>69.3293mm</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>47.3525mm</t>
+          <t>24.7650mm</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -2059,24 +2059,24 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>270</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>C64</t>
+          <t>C65</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>69.3293mm</t>
+          <t>98.2750mm</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>24.7650mm</t>
+          <t>38.4900mm</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -2086,24 +2086,24 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>C65</t>
+          <t>C66</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>98.2750mm</t>
+          <t>87.6250mm</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>38.4900mm</t>
+          <t>46.5900mm</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -2113,19 +2113,19 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>270</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>C66</t>
+          <t>C67</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>87.6250mm</t>
+          <t>89.2250mm</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2140,24 +2140,24 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>C67</t>
+          <t>C68</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>89.2250mm</t>
+          <t>87.6250mm</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>46.5900mm</t>
+          <t>43.4400mm</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2167,24 +2167,24 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>270</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>C68</t>
+          <t>C69</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>87.6250mm</t>
+          <t>93.2250mm</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>43.4400mm</t>
+          <t>9.9700mm</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2194,24 +2194,24 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>C69</t>
+          <t>C7</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>93.2250mm</t>
+          <t>80.1456mm</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>9.9700mm</t>
+          <t>14.4900mm</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2228,17 +2228,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>C7</t>
+          <t>C70</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>80.1456mm</t>
+          <t>69.0000mm</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>14.4900mm</t>
+          <t>34.0000mm</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2248,19 +2248,19 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>270</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>C70</t>
+          <t>C71</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>69.0000mm</t>
+          <t>75.0000mm</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -2275,24 +2275,24 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>C71</t>
+          <t>C72</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>75.0000mm</t>
+          <t>17.4625mm</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>34.0000mm</t>
+          <t>7.9375mm</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2302,24 +2302,24 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>270</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>C72</t>
+          <t>C73</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>17.7800mm</t>
+          <t>36.5125mm</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>7.9375mm</t>
+          <t>21.2725mm</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2329,19 +2329,19 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>C73</t>
+          <t>C74</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>36.5125mm</t>
+          <t>39.3700mm</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -2363,17 +2363,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>C74</t>
+          <t>C8</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>39.3700mm</t>
+          <t>92.2750mm</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>21.2725mm</t>
+          <t>16.6900mm</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2383,24 +2383,24 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>180</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>C8</t>
+          <t>C9</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>92.2750mm</t>
+          <t>95.3750mm</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>16.6900mm</t>
+          <t>18.4400mm</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2410,24 +2410,24 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>270</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>C9</t>
+          <t>IC1</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>95.3750mm</t>
+          <t>72.0000mm</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>18.4400mm</t>
+          <t>11.0000mm</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2444,7 +2444,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>IC1</t>
+          <t>IC2</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2454,7 +2454,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>11.0000mm</t>
+          <t>34.0000mm</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2471,17 +2471,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>IC2</t>
+          <t>IC3</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>72.0000mm</t>
+          <t>56.7817mm</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>34.0000mm</t>
+          <t>8.9789mm</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2491,24 +2491,24 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>180</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>IC3</t>
+          <t>IC4</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>56.7817mm</t>
+          <t>43.4975mm</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>8.9789mm</t>
+          <t>7.9375mm</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2525,17 +2525,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>IC4</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>43.4975mm</t>
+          <t>92.4034mm</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>7.9375mm</t>
+          <t>30.3231mm</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2552,17 +2552,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>92.4034mm</t>
+          <t>78.3458mm</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>30.3231mm</t>
+          <t>34.2487mm</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -2572,24 +2572,24 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L27</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>78.3458mm</t>
+          <t>98.2302mm</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>34.2487mm</t>
+          <t>19.1053mm</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -2599,24 +2599,24 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>L27</t>
+          <t>L3</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>98.2302mm</t>
+          <t>77.9388mm</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>19.1053mm</t>
+          <t>38.8156mm</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2626,24 +2626,24 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>L3</t>
+          <t>L30</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>77.9388mm</t>
+          <t>78.3458mm</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>38.8156mm</t>
+          <t>10.2487mm</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2660,17 +2660,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>L30</t>
+          <t>L31</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>78.3458mm</t>
+          <t>77.9388mm</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>10.2487mm</t>
+          <t>14.8156mm</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2687,17 +2687,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>L31</t>
+          <t>L32</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>77.9388mm</t>
+          <t>92.4034mm</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>14.8156mm</t>
+          <t>6.3231mm</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2707,24 +2707,24 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>180</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>L32</t>
+          <t>L4</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>92.4034mm</t>
+          <t>98.2810mm</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>6.3231mm</t>
+          <t>43.1815mm</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2734,24 +2734,24 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>L4</t>
+          <t>L5</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>98.2810mm</t>
+          <t>20.0025mm</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>43.1815mm</t>
+          <t>13.6525mm</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2768,17 +2768,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>L5</t>
+          <t>L6</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>20.0025mm</t>
+          <t>67.9450mm</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>13.6525mm</t>
+          <t>27.3050mm</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -2795,12 +2795,12 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>L6</t>
+          <t>L7</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>67.9450mm</t>
+          <t>70.9549mm</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -2822,17 +2822,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>L7</t>
+          <t>L8</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>70.9549mm</t>
+          <t>58.8164mm</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>27.3050mm</t>
+          <t>14.2452mm</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -2842,24 +2842,24 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>L8</t>
+          <t>L9</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>58.8164mm</t>
+          <t>73.9775mm</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>14.2452mm</t>
+          <t>27.3050mm</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -2869,24 +2869,24 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>L9</t>
+          <t>LED1</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>73.9775mm</t>
+          <t>51.1175mm</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>27.3050mm</t>
+          <t>39.0525mm</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -2903,12 +2903,12 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>LED1</t>
+          <t>LED2</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>51.1175mm</t>
+          <t>43.4975mm</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -2930,12 +2930,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>LED2</t>
+          <t>LED3</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>43.4975mm</t>
+          <t>40.9575mm</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -2957,12 +2957,12 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>LED3</t>
+          <t>LED4</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>40.9575mm</t>
+          <t>48.5775mm</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -2984,49 +2984,49 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>LED4</t>
+          <t>OSC1</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>48.5775mm</t>
+          <t>65.2800mm</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>39.0525mm</t>
+          <t>14.4875mm</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>270</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>OSC1</t>
+          <t>PS1</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>65.2800mm</t>
+          <t>9.8425mm</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>14.4875mm</t>
+          <t>17.4625mm</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -3038,17 +3038,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>PS1</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>9.8425mm</t>
+          <t>85.9750mm</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>17.4625mm</t>
+          <t>19.4400mm</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -3058,24 +3058,24 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R10</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>85.9750mm</t>
+          <t>95.3250mm</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>19.4400mm</t>
+          <t>39.3900mm</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -3092,17 +3092,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>R10</t>
+          <t>R11</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>95.3250mm</t>
+          <t>62.0649mm</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>39.3900mm</t>
+          <t>7.8613mm</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -3112,24 +3112,24 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>R11</t>
+          <t>R12</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>62.0649mm</t>
+          <t>78.4225mm</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>7.8613mm</t>
+          <t>23.8125mm</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -3139,24 +3139,24 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>180</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>R12</t>
+          <t>R13</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>78.4225mm</t>
+          <t>68.1101mm</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>23.8125mm</t>
+          <t>22.2250mm</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -3173,17 +3173,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>R13</t>
+          <t>R14</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>68.1101mm</t>
+          <t>9.2075mm</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>22.2250mm</t>
+          <t>6.3500mm</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -3193,24 +3193,24 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>270</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>R14</t>
+          <t>R15</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>9.2075mm</t>
+          <t>35.2425mm</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>6.3500mm</t>
+          <t>14.9225mm</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -3227,7 +3227,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>R15</t>
+          <t>R16</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -3237,7 +3237,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>14.9225mm</t>
+          <t>10.7950mm</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -3254,17 +3254,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>R16</t>
+          <t>R17</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>35.2425mm</t>
+          <t>6.9850mm</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>10.7950mm</t>
+          <t>6.3500mm</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -3274,24 +3274,24 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>R17</t>
+          <t>R18</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>6.9850mm</t>
+          <t>51.1175mm</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>6.3500mm</t>
+          <t>35.8775mm</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -3301,19 +3301,19 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>270</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>R18</t>
+          <t>R19</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>51.1175mm</t>
+          <t>43.4975mm</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -3335,17 +3335,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>R19</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>43.4975mm</t>
+          <t>85.7412mm</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>35.8775mm</t>
+          <t>7.6172mm</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -3362,17 +3362,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>R20</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>85.7412mm</t>
+          <t>40.9575mm</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>7.6172mm</t>
+          <t>35.8775mm</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -3389,17 +3389,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>R20</t>
+          <t>R21</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>40.9575mm</t>
+          <t>48.5775mm</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>35.8775mm</t>
+          <t>35.5600mm</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -3416,17 +3416,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>R21</t>
+          <t>R22</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>48.5775mm</t>
+          <t>9.2075mm</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>35.5600mm</t>
+          <t>44.7675mm</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -3436,24 +3436,24 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>R22</t>
+          <t>R23</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>9.2075mm</t>
+          <t>13.9700mm</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>44.7675mm</t>
+          <t>40.6400mm</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -3463,24 +3463,24 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>180</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>R23</t>
+          <t>R24</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>13.9700mm</t>
+          <t>27.9400mm</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>40.6400mm</t>
+          <t>42.2275mm</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -3497,17 +3497,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>R24</t>
+          <t>R25</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>27.9400mm</t>
+          <t>19.3675mm</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>42.2275mm</t>
+          <t>43.1800mm</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -3524,17 +3524,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>R25</t>
+          <t>R26</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>19.3675mm</t>
+          <t>65.0875mm</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>43.1800mm</t>
+          <t>22.2250mm</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -3544,24 +3544,24 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>R26</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>65.0875mm</t>
+          <t>85.9750mm</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>22.2250mm</t>
+          <t>43.4400mm</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -3571,24 +3571,24 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R34</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>85.9750mm</t>
+          <t>90.8750mm</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>43.4400mm</t>
+          <t>22.5900mm</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -3598,24 +3598,24 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>270</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>R34</t>
+          <t>R35</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>90.8750mm</t>
+          <t>89.2250mm</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>22.5900mm</t>
+          <t>19.4400mm</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -3625,24 +3625,24 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>R35</t>
+          <t>R36</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>89.2250mm</t>
+          <t>92.5250mm</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>19.4400mm</t>
+          <t>22.5900mm</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -3652,19 +3652,19 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>270</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>R36</t>
+          <t>R37</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>92.5250mm</t>
+          <t>94.2250mm</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -3679,24 +3679,24 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>R37</t>
+          <t>R38</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>94.2250mm</t>
+          <t>95.3592mm</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>22.5900mm</t>
+          <t>11.6990mm</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -3706,24 +3706,24 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>270</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>R38</t>
+          <t>R39</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>95.3592mm</t>
+          <t>95.3250mm</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>11.6990mm</t>
+          <t>15.3900mm</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -3733,24 +3733,24 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>R39</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>95.3250mm</t>
+          <t>85.7412mm</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>15.3900mm</t>
+          <t>31.6172mm</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -3760,24 +3760,24 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>270</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R5</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>85.7412mm</t>
+          <t>90.8750mm</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>31.6172mm</t>
+          <t>46.5900mm</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -3794,17 +3794,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R6</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>90.8750mm</t>
+          <t>89.2250mm</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>46.5900mm</t>
+          <t>43.4400mm</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -3814,24 +3814,24 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>R6</t>
+          <t>R7</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>89.2250mm</t>
+          <t>92.5250mm</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>43.4400mm</t>
+          <t>46.5900mm</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -3841,19 +3841,19 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>270</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R8</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>92.5250mm</t>
+          <t>94.2250mm</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -3868,24 +3868,24 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>R8</t>
+          <t>R9</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>94.2250mm</t>
+          <t>95.3592mm</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>46.5900mm</t>
+          <t>35.6990mm</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -3895,24 +3895,24 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>270</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>R9</t>
+          <t>SCK1</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>95.3592mm</t>
+          <t>108.0000mm</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>35.6990mm</t>
+          <t>14.0000mm</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -3922,24 +3922,24 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>180</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>SCK1</t>
+          <t>SCK2</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>108.0000mm</t>
+          <t>107.7980mm</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>14.0000mm</t>
+          <t>38.3630mm</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -3956,17 +3956,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>SCK2</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>107.7980mm</t>
+          <t>13.3350mm</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>38.3630mm</t>
+          <t>43.8150mm</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -3976,24 +3976,24 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>270</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>TR4</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>13.3350mm</t>
+          <t>23.1775mm</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>43.8150mm</t>
+          <t>42.2275mm</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -4010,22 +4010,22 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>TR4</t>
+          <t>U$2</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>23.1775mm</t>
+          <t>25.7175mm</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>42.2275mm</t>
+          <t>27.6225mm</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
@@ -4037,17 +4037,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>U$2</t>
+          <t>U1</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>25.7175mm</t>
+          <t>26.9875mm</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>27.6225mm</t>
+          <t>40.3225mm</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -4064,34 +4064,34 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>U2</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>26.9875mm</t>
+          <t>87.0750mm</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>40.3225mm</t>
+          <t>13.6400mm</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>U2</t>
+          <t>U3</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -4101,7 +4101,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>13.6400mm</t>
+          <t>37.6400mm</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -4110,33 +4110,6 @@
         </is>
       </c>
       <c r="E137" t="inlineStr">
-        <is>
-          <t>90</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" t="inlineStr">
-        <is>
-          <t>U3</t>
-        </is>
-      </c>
-      <c r="B138" t="inlineStr">
-        <is>
-          <t>87.0750mm</t>
-        </is>
-      </c>
-      <c r="C138" t="inlineStr">
-        <is>
-          <t>37.6400mm</t>
-        </is>
-      </c>
-      <c r="D138" t="inlineStr">
-        <is>
-          <t>Top</t>
-        </is>
-      </c>
-      <c r="E138" t="inlineStr">
         <is>
           <t>90</t>
         </is>

</xml_diff>